<commit_message>
benchmarking data and rereunning at multiple thresholds
</commit_message>
<xml_diff>
--- a/10_Threshold_OUTPUT/direct_A0A072Z841_Corynebacterium_glutamicum_ATCC_13032.xlsx
+++ b/10_Threshold_OUTPUT/direct_A0A072Z841_Corynebacterium_glutamicum_ATCC_13032.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,15 +446,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>full_pattern</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>group1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>group2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>full_pattern_html</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
@@ -477,15 +487,25 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>TCGAACATATGTTCGA</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>TCGA</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>TCGA</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>&lt;span style="color: red; font-weight: bold;"&gt;T&lt;/span&gt;&lt;span style="color: red; font-weight: bold;"&gt;C&lt;/span&gt;&lt;span style="color: red; font-weight: bold;"&gt;G&lt;/span&gt;&lt;span style="color: red; font-weight: bold;"&gt;A&lt;/span&gt;ACATATGT&lt;span style="color: blue; font-weight: bold;"&gt;T&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;C&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;G&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;A&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
         <v>0.07077169132347061</v>
       </c>
     </row>
@@ -506,15 +526,25 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>AACA</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>ACA</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>&lt;span style="color: red; font-weight: bold;"&gt;A&lt;/span&gt;&lt;span style="color: purple; font-weight: bold;"&gt;A&lt;/span&gt;&lt;span style="color: purple; font-weight: bold;"&gt;C&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;A&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
         <v>0.7714914034386245</v>
       </c>
     </row>
@@ -535,15 +565,25 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>AACA</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>&lt;span style="color: red; font-weight: bold;"&gt;A&lt;/span&gt;&lt;span style="color: red; font-weight: bold;"&gt;A&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;C&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;A&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
         <v>0.9218312674930028</v>
       </c>
     </row>
@@ -564,15 +604,25 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>TGTTCG</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>CG</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>TG</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>&lt;span style="color: red; font-weight: bold;"&gt;T&lt;/span&gt;&lt;span style="color: red; font-weight: bold;"&gt;G&lt;/span&gt;TT&lt;span style="color: blue; font-weight: bold;"&gt;C&lt;/span&gt;&lt;span style="color: blue; font-weight: bold;"&gt;G&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>0.9994002399040384</v>
       </c>
     </row>

</xml_diff>